<commit_message>
Fixed mass flow out of orifice
</commit_message>
<xml_diff>
--- a/data/fill_inputs.xlsx
+++ b/data/fill_inputs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gbhof\Documents\SARP\Code\Sim Matalb\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db8d08c81090d50f/Documents/MATLAB/Fill-Simulator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F3C89C-E450-4355-94DD-70CE06ED0FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{30F3C89C-E450-4355-94DD-70CE06ED0FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04FC0C47-9BAE-412C-99C4-1C6F9020EC33}"/>
   <bookViews>
-    <workbookView xWindow="5235" yWindow="4043" windowWidth="18225" windowHeight="11332" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>PARAMETER</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>Run Tank Volume (ft3)</t>
+  </si>
+  <si>
+    <t>Atmospheric Pressure (psia)</t>
   </si>
 </sst>
 </file>
@@ -378,13 +381,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.86328125" customWidth="1"/>
+    <col min="1" max="1" width="25.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -392,7 +395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -400,7 +403,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -408,7 +411,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -416,7 +419,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -424,7 +427,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -432,7 +435,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -440,12 +443,20 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8">
         <v>0.32986100000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>14.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added holding sim abilities, attempted to implement heat transfer
</commit_message>
<xml_diff>
--- a/data/fill_inputs.xlsx
+++ b/data/fill_inputs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/db8d08c81090d50f/Documents/MATLAB/Fill-Simulator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{30F3C89C-E450-4355-94DD-70CE06ED0FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04FC0C47-9BAE-412C-99C4-1C6F9020EC33}"/>
+  <xr:revisionPtr revIDLastSave="91" documentId="13_ncr:1_{30F3C89C-E450-4355-94DD-70CE06ED0FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{500BDDE8-36EF-48DF-A056-657B1105C526}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>PARAMETER</t>
   </si>
@@ -55,6 +55,30 @@
   </si>
   <si>
     <t>Atmospheric Pressure (psia)</t>
+  </si>
+  <si>
+    <t>Timestep</t>
+  </si>
+  <si>
+    <t>Internal Surface Area of Run Tank (m^2)</t>
+  </si>
+  <si>
+    <t>Heat Transfer Coefficient for Nitrous</t>
+  </si>
+  <si>
+    <t>Solar Zenith (degrees)</t>
+  </si>
+  <si>
+    <t>Wind Speed (mph)</t>
+  </si>
+  <si>
+    <t>Specific Heat of Aluminum (Cp)</t>
+  </si>
+  <si>
+    <t>Mass of Run Tank (kg)</t>
+  </si>
+  <si>
+    <t>External Surface Area of Run Tank (m^2)</t>
   </si>
 </sst>
 </file>
@@ -98,9 +122,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -116,6 +143,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -381,10 +412,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -408,7 +440,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -416,7 +448,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.01</v>
+        <v>2.1000000000000001E-2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -459,7 +491,72 @@
         <v>14.7</v>
       </c>
     </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>0.234896304</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
+        <v>0.25839948299999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>9.07</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>